<commit_message>
chore: checkpoint workspace changes
</commit_message>
<xml_diff>
--- a/mts/DP2-PIAGET.xlsx
+++ b/mts/DP2-PIAGET.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="208">
   <si>
     <t>Attribute</t>
   </si>
@@ -144,10 +144,7 @@
     <t>pmsr:INI1784879596190461</t>
   </si>
   <si>
-    <t>2025-06-05T13:01:01.000</t>
-  </si>
-  <si>
-    <t>2025-06-05T13:01:02.000</t>
+    <t>2024-01-01</t>
   </si>
   <si>
     <t>pmsr:DPL1784879596777301</t>
@@ -363,7 +360,7 @@
     <t>hasco:partOf</t>
   </si>
   <si>
-    <t>vstoi:Platform</t>
+    <t>vstoi:Laboratory</t>
   </si>
   <si>
     <t>Laboratório de Prática Simulada I</t>
@@ -432,6 +429,12 @@
     <t>080001</t>
   </si>
   <si>
+    <t>Low fidelity mannequin</t>
+  </si>
+  <si>
+    <t>Nursing Anne Basic</t>
+  </si>
+  <si>
     <t>Low-Fidelity Mannequin. SN: 080002</t>
   </si>
   <si>
@@ -459,6 +462,12 @@
     <t>080005</t>
   </si>
   <si>
+    <t>High fidelity full body simulator</t>
+  </si>
+  <si>
+    <t>Nursing Anne Simulator</t>
+  </si>
+  <si>
     <t>pmsr:/INS1739397556188145</t>
   </si>
   <si>
@@ -468,24 +477,45 @@
     <t>080006</t>
   </si>
   <si>
+    <t>Advanced Life Support adult mannequin</t>
+  </si>
+  <si>
+    <t>Resusci Anne Simulator</t>
+  </si>
+  <si>
     <t>Laerdal Nursing Anne Mannequin. SN: 090001</t>
   </si>
   <si>
     <t>090001</t>
   </si>
   <si>
+    <t>Gaia CSPC - High fidelity simulator</t>
+  </si>
+  <si>
+    <t>Nursing Anne</t>
+  </si>
+  <si>
     <t>Laerdal Nursing Anne Mannequin. SN: 090002</t>
   </si>
   <si>
     <t>090002</t>
   </si>
   <si>
+    <t>Resusci Anne</t>
+  </si>
+  <si>
     <t>Low-Fidelity Mannequin. SN: 090003</t>
   </si>
   <si>
     <t>090003</t>
   </si>
   <si>
+    <t>Gaia LPE1 - Low fidelity mannequin</t>
+  </si>
+  <si>
+    <t>Basic Mannequin</t>
+  </si>
+  <si>
     <t>Low-Fidelity Mannequin. SN: 090004</t>
   </si>
   <si>
@@ -510,6 +540,9 @@
     <t>090007</t>
   </si>
   <si>
+    <t>Gaia LPE2 - Low fidelity mannequin</t>
+  </si>
+  <si>
     <t>Low-Fidelity Mannequin. SN: 090008</t>
   </si>
   <si>
@@ -534,10 +567,16 @@
     <t>100001</t>
   </si>
   <si>
+    <t>Full body medium tone simulator with articulated limbs</t>
+  </si>
+  <si>
     <t>Gynaecological Examination Mannequin. SN: 100002</t>
   </si>
   <si>
     <t>100002</t>
+  </si>
+  <si>
+    <t>Emergency intervention training simulator</t>
   </si>
   <si>
     <t>vstoi:isInstrumentAttachment</t>
@@ -644,7 +683,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -727,28 +766,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -779,19 +803,10 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
@@ -2571,10 +2586,10 @@
       <c r="F1" t="s" s="2">
         <v>32</v>
       </c>
-      <c r="G1" t="s" s="5">
+      <c r="G1" t="s" s="2">
         <v>33</v>
       </c>
-      <c r="H1" t="s" s="5">
+      <c r="H1" t="s" s="2">
         <v>34</v>
       </c>
       <c r="I1" t="s" s="2">
@@ -2616,14 +2631,12 @@
       <c r="E2" t="s" s="2">
         <v>40</v>
       </c>
-      <c r="F2" s="10"/>
-      <c r="G2" t="s" s="6">
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H2" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I2" s="7"/>
+      <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
@@ -2646,28 +2659,26 @@
     </row>
     <row r="3" ht="13.55" customHeight="1">
       <c r="A3" t="s" s="2">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D3" t="s" s="2">
         <v>39</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>45</v>
-      </c>
-      <c r="F3" s="10"/>
-      <c r="G3" t="s" s="6">
+        <v>44</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H3" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I3" s="7"/>
+      <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
@@ -2690,28 +2701,26 @@
     </row>
     <row r="4" ht="13.55" customHeight="1">
       <c r="A4" t="s" s="2">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B4" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D4" t="s" s="2">
         <v>39</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>48</v>
-      </c>
-      <c r="F4" s="10"/>
-      <c r="G4" t="s" s="6">
+        <v>47</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H4" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I4" s="7"/>
+      <c r="I4" s="3"/>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
@@ -2734,28 +2743,26 @@
     </row>
     <row r="5" ht="13.55" customHeight="1">
       <c r="A5" t="s" s="2">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B5" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C5" t="s" s="2">
+        <v>49</v>
+      </c>
+      <c r="D5" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="D5" t="s" s="2">
+      <c r="E5" t="s" s="2">
         <v>51</v>
       </c>
-      <c r="E5" t="s" s="2">
-        <v>52</v>
-      </c>
-      <c r="F5" s="10"/>
-      <c r="G5" t="s" s="6">
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H5" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I5" s="7"/>
+      <c r="I5" s="3"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
@@ -2778,28 +2785,26 @@
     </row>
     <row r="6" ht="13.55" customHeight="1">
       <c r="A6" t="s" s="2">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B6" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C6" t="s" s="2">
+        <v>53</v>
+      </c>
+      <c r="D6" t="s" s="2">
         <v>54</v>
       </c>
-      <c r="D6" t="s" s="2">
+      <c r="E6" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="E6" t="s" s="2">
-        <v>56</v>
-      </c>
-      <c r="F6" s="10"/>
-      <c r="G6" t="s" s="6">
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H6" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I6" s="7"/>
+      <c r="I6" s="3"/>
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
@@ -2822,28 +2827,26 @@
     </row>
     <row r="7" ht="13.55" customHeight="1">
       <c r="A7" t="s" s="2">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B7" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C7" t="s" s="2">
+        <v>57</v>
+      </c>
+      <c r="D7" t="s" s="2">
+        <v>54</v>
+      </c>
+      <c r="E7" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="D7" t="s" s="2">
-        <v>55</v>
-      </c>
-      <c r="E7" t="s" s="2">
-        <v>59</v>
-      </c>
-      <c r="F7" s="10"/>
-      <c r="G7" t="s" s="6">
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H7" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I7" s="7"/>
+      <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
       <c r="L7" s="3"/>
@@ -2866,28 +2869,26 @@
     </row>
     <row r="8" ht="13.55" customHeight="1">
       <c r="A8" t="s" s="2">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B8" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C8" t="s" s="2">
+        <v>60</v>
+      </c>
+      <c r="D8" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="D8" t="s" s="2">
+      <c r="E8" t="s" s="2">
         <v>62</v>
       </c>
-      <c r="E8" t="s" s="2">
-        <v>63</v>
-      </c>
-      <c r="F8" s="10"/>
-      <c r="G8" t="s" s="6">
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H8" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I8" s="7"/>
+      <c r="I8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
       <c r="L8" s="3"/>
@@ -2910,28 +2911,26 @@
     </row>
     <row r="9" ht="13.55" customHeight="1">
       <c r="A9" t="s" s="2">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B9" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C9" t="s" s="2">
+        <v>64</v>
+      </c>
+      <c r="D9" t="s" s="2">
+        <v>61</v>
+      </c>
+      <c r="E9" t="s" s="2">
         <v>65</v>
       </c>
-      <c r="D9" t="s" s="2">
-        <v>62</v>
-      </c>
-      <c r="E9" t="s" s="2">
-        <v>66</v>
-      </c>
-      <c r="F9" s="10"/>
-      <c r="G9" t="s" s="6">
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H9" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I9" s="7"/>
+      <c r="I9" s="3"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
@@ -2954,28 +2953,26 @@
     </row>
     <row r="10" ht="13.55" customHeight="1">
       <c r="A10" t="s" s="2">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B10" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C10" t="s" s="2">
+        <v>67</v>
+      </c>
+      <c r="D10" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="D10" t="s" s="2">
+      <c r="E10" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="E10" t="s" s="2">
-        <v>70</v>
-      </c>
-      <c r="F10" s="10"/>
-      <c r="G10" t="s" s="6">
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H10" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I10" s="7"/>
+      <c r="I10" s="3"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
@@ -2998,28 +2995,26 @@
     </row>
     <row r="11" ht="13.55" customHeight="1">
       <c r="A11" t="s" s="2">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B11" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C11" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="D11" t="s" s="2">
+        <v>68</v>
+      </c>
+      <c r="E11" t="s" s="2">
         <v>72</v>
       </c>
-      <c r="D11" t="s" s="2">
-        <v>69</v>
-      </c>
-      <c r="E11" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="F11" s="10"/>
-      <c r="G11" t="s" s="6">
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H11" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I11" s="7"/>
+      <c r="I11" s="3"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
@@ -3042,28 +3037,26 @@
     </row>
     <row r="12" ht="13.55" customHeight="1">
       <c r="A12" t="s" s="2">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B12" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C12" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="D12" t="s" s="2">
+        <v>68</v>
+      </c>
+      <c r="E12" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="D12" t="s" s="2">
-        <v>69</v>
-      </c>
-      <c r="E12" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="F12" s="10"/>
-      <c r="G12" t="s" s="6">
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H12" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I12" s="7"/>
+      <c r="I12" s="3"/>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
@@ -3086,28 +3079,26 @@
     </row>
     <row r="13" ht="13.55" customHeight="1">
       <c r="A13" t="s" s="2">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B13" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C13" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="D13" t="s" s="2">
+        <v>68</v>
+      </c>
+      <c r="E13" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="D13" t="s" s="2">
-        <v>69</v>
-      </c>
-      <c r="E13" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="F13" s="10"/>
-      <c r="G13" t="s" s="6">
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H13" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I13" s="7"/>
+      <c r="I13" s="3"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
@@ -3130,28 +3121,26 @@
     </row>
     <row r="14" ht="13.55" customHeight="1">
       <c r="A14" t="s" s="2">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B14" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C14" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="D14" t="s" s="2">
         <v>81</v>
       </c>
-      <c r="D14" t="s" s="2">
+      <c r="E14" t="s" s="2">
         <v>82</v>
       </c>
-      <c r="E14" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="F14" s="10"/>
-      <c r="G14" t="s" s="6">
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H14" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I14" s="7"/>
+      <c r="I14" s="3"/>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
       <c r="L14" s="3"/>
@@ -3174,28 +3163,26 @@
     </row>
     <row r="15" ht="13.55" customHeight="1">
       <c r="A15" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B15" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C15" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="D15" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E15" t="s" s="2">
         <v>85</v>
       </c>
-      <c r="D15" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E15" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="F15" s="10"/>
-      <c r="G15" t="s" s="6">
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H15" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I15" s="7"/>
+      <c r="I15" s="3"/>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
@@ -3218,28 +3205,26 @@
     </row>
     <row r="16" ht="13.55" customHeight="1">
       <c r="A16" t="s" s="2">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B16" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C16" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="D16" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E16" t="s" s="2">
         <v>88</v>
       </c>
-      <c r="D16" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E16" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="F16" s="10"/>
-      <c r="G16" t="s" s="6">
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H16" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I16" s="7"/>
+      <c r="I16" s="3"/>
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
       <c r="L16" s="3"/>
@@ -3262,28 +3247,26 @@
     </row>
     <row r="17" ht="13.55" customHeight="1">
       <c r="A17" t="s" s="2">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B17" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C17" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="D17" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E17" t="s" s="2">
         <v>91</v>
       </c>
-      <c r="D17" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E17" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="F17" s="10"/>
-      <c r="G17" t="s" s="6">
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H17" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I17" s="7"/>
+      <c r="I17" s="3"/>
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
       <c r="L17" s="3"/>
@@ -3306,28 +3289,26 @@
     </row>
     <row r="18" ht="13.55" customHeight="1">
       <c r="A18" t="s" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B18" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C18" t="s" s="2">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D18" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="E18" t="s" s="2">
         <v>94</v>
       </c>
-      <c r="E18" t="s" s="2">
-        <v>95</v>
-      </c>
-      <c r="F18" s="10"/>
-      <c r="G18" t="s" s="6">
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H18" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I18" s="7"/>
+      <c r="I18" s="3"/>
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
       <c r="L18" s="3"/>
@@ -3350,28 +3331,26 @@
     </row>
     <row r="19" ht="13.55" customHeight="1">
       <c r="A19" t="s" s="2">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B19" t="s" s="2">
         <v>37</v>
       </c>
       <c r="C19" t="s" s="2">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D19" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E19" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="F19" s="10"/>
-      <c r="G19" t="s" s="6">
+        <v>96</v>
+      </c>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="H19" t="s" s="6">
-        <v>42</v>
-      </c>
-      <c r="I19" s="7"/>
+      <c r="I19" s="3"/>
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
@@ -3406,8 +3385,8 @@
   <dimension ref="A1:G10"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="7" width="8.85156" style="11" customWidth="1"/>
-    <col min="8" max="16384" width="8.85156" style="11" customWidth="1"/>
+    <col min="1" max="7" width="8.85156" style="10" customWidth="1"/>
+    <col min="8" max="16384" width="8.85156" style="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.55" customHeight="1">
@@ -3415,22 +3394,22 @@
         <v>27</v>
       </c>
       <c r="B1" t="s" s="2">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C1" t="s" s="2">
         <v>29</v>
       </c>
       <c r="D1" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="E1" t="s" s="2">
         <v>99</v>
       </c>
-      <c r="E1" t="s" s="2">
+      <c r="F1" t="s" s="2">
         <v>100</v>
       </c>
-      <c r="F1" t="s" s="2">
+      <c r="G1" t="s" s="2">
         <v>101</v>
-      </c>
-      <c r="G1" t="s" s="2">
-        <v>102</v>
       </c>
     </row>
     <row r="2" ht="13.55" customHeight="1">
@@ -3528,63 +3507,63 @@
   <dimension ref="A1:Z11"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="26" style="12" customWidth="1"/>
-    <col min="2" max="2" width="24" style="12" customWidth="1"/>
-    <col min="3" max="3" width="33" style="12" customWidth="1"/>
-    <col min="4" max="4" width="25.8516" style="12" customWidth="1"/>
-    <col min="5" max="5" width="23.5" style="12" customWidth="1"/>
-    <col min="6" max="6" width="15.6719" style="12" customWidth="1"/>
-    <col min="7" max="7" width="16.5" style="12" customWidth="1"/>
-    <col min="8" max="8" width="9.5" style="12" customWidth="1"/>
-    <col min="9" max="12" width="8.85156" style="12" customWidth="1"/>
-    <col min="13" max="13" width="9.67188" style="12" customWidth="1"/>
-    <col min="14" max="14" width="28" style="12" customWidth="1"/>
-    <col min="15" max="26" width="8.85156" style="12" customWidth="1"/>
-    <col min="27" max="16384" width="8.85156" style="12" customWidth="1"/>
+    <col min="1" max="1" width="26" style="11" customWidth="1"/>
+    <col min="2" max="2" width="24" style="11" customWidth="1"/>
+    <col min="3" max="3" width="33" style="11" customWidth="1"/>
+    <col min="4" max="4" width="25.8516" style="11" customWidth="1"/>
+    <col min="5" max="5" width="23.5" style="11" customWidth="1"/>
+    <col min="6" max="6" width="15.6719" style="11" customWidth="1"/>
+    <col min="7" max="7" width="16.5" style="11" customWidth="1"/>
+    <col min="8" max="8" width="9.5" style="11" customWidth="1"/>
+    <col min="9" max="12" width="8.85156" style="11" customWidth="1"/>
+    <col min="13" max="13" width="9.67188" style="11" customWidth="1"/>
+    <col min="14" max="14" width="28" style="11" customWidth="1"/>
+    <col min="15" max="26" width="8.85156" style="11" customWidth="1"/>
+    <col min="27" max="16384" width="8.85156" style="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.55" customHeight="1">
       <c r="A1" t="s" s="2">
         <v>27</v>
       </c>
-      <c r="B1" t="s" s="5">
+      <c r="B1" t="s" s="2">
         <v>28</v>
       </c>
       <c r="C1" t="s" s="2">
         <v>29</v>
       </c>
       <c r="D1" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="E1" t="s" s="2">
         <v>103</v>
       </c>
-      <c r="E1" t="s" s="2">
+      <c r="F1" t="s" s="2">
         <v>104</v>
       </c>
-      <c r="F1" t="s" s="2">
+      <c r="G1" t="s" s="2">
         <v>105</v>
       </c>
-      <c r="G1" t="s" s="2">
+      <c r="H1" t="s" s="2">
         <v>106</v>
       </c>
-      <c r="H1" t="s" s="2">
+      <c r="I1" t="s" s="2">
         <v>107</v>
       </c>
-      <c r="I1" t="s" s="2">
+      <c r="J1" t="s" s="2">
         <v>108</v>
       </c>
-      <c r="J1" t="s" s="2">
+      <c r="K1" t="s" s="2">
         <v>109</v>
       </c>
-      <c r="K1" t="s" s="2">
+      <c r="L1" t="s" s="2">
         <v>110</v>
       </c>
-      <c r="L1" t="s" s="2">
+      <c r="M1" t="s" s="2">
         <v>111</v>
       </c>
-      <c r="M1" t="s" s="2">
+      <c r="N1" t="s" s="2">
         <v>112</v>
-      </c>
-      <c r="N1" t="s" s="2">
-        <v>113</v>
       </c>
       <c r="O1" s="3"/>
       <c r="P1" s="3"/>
@@ -3600,14 +3579,14 @@
       <c r="Z1" s="3"/>
     </row>
     <row r="2" ht="13.55" customHeight="1">
-      <c r="A2" t="s" s="13">
+      <c r="A2" t="s" s="2">
         <v>39</v>
       </c>
-      <c r="B2" t="s" s="6">
+      <c r="B2" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="C2" t="s" s="2">
         <v>114</v>
-      </c>
-      <c r="C2" t="s" s="14">
-        <v>115</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
@@ -3620,7 +3599,7 @@
       <c r="L2" s="3"/>
       <c r="M2" s="3"/>
       <c r="N2" t="s" s="2">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
@@ -3636,14 +3615,14 @@
       <c r="Z2" s="3"/>
     </row>
     <row r="3" ht="13.55" customHeight="1">
-      <c r="A3" t="s" s="13">
-        <v>51</v>
-      </c>
-      <c r="B3" t="s" s="6">
-        <v>114</v>
-      </c>
-      <c r="C3" t="s" s="14">
-        <v>117</v>
+      <c r="A3" t="s" s="2">
+        <v>50</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="C3" t="s" s="2">
+        <v>116</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
@@ -3656,7 +3635,7 @@
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
       <c r="N3" t="s" s="2">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
@@ -3672,14 +3651,14 @@
       <c r="Z3" s="3"/>
     </row>
     <row r="4" ht="13.55" customHeight="1">
-      <c r="A4" t="s" s="13">
-        <v>55</v>
-      </c>
-      <c r="B4" t="s" s="6">
-        <v>114</v>
-      </c>
-      <c r="C4" t="s" s="14">
-        <v>118</v>
+      <c r="A4" t="s" s="2">
+        <v>54</v>
+      </c>
+      <c r="B4" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="C4" t="s" s="2">
+        <v>117</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -3692,7 +3671,7 @@
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
       <c r="N4" t="s" s="2">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
@@ -3708,14 +3687,14 @@
       <c r="Z4" s="3"/>
     </row>
     <row r="5" ht="13.55" customHeight="1">
-      <c r="A5" t="s" s="13">
+      <c r="A5" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="B5" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="C5" t="s" s="2">
         <v>119</v>
-      </c>
-      <c r="B5" t="s" s="6">
-        <v>114</v>
-      </c>
-      <c r="C5" t="s" s="14">
-        <v>120</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
@@ -3728,7 +3707,7 @@
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
       <c r="N5" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="O5" s="3"/>
       <c r="P5" s="3"/>
@@ -3744,14 +3723,14 @@
       <c r="Z5" s="3"/>
     </row>
     <row r="6" ht="13.55" customHeight="1">
-      <c r="A6" t="s" s="13">
+      <c r="A6" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="B6" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="C6" t="s" s="2">
         <v>122</v>
-      </c>
-      <c r="B6" t="s" s="6">
-        <v>114</v>
-      </c>
-      <c r="C6" t="s" s="14">
-        <v>123</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
@@ -3764,7 +3743,7 @@
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
       <c r="N6" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="O6" s="3"/>
       <c r="P6" s="3"/>
@@ -3780,14 +3759,14 @@
       <c r="Z6" s="3"/>
     </row>
     <row r="7" ht="13.55" customHeight="1">
-      <c r="A7" t="s" s="13">
+      <c r="A7" t="s" s="2">
+        <v>123</v>
+      </c>
+      <c r="B7" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="C7" t="s" s="2">
         <v>124</v>
-      </c>
-      <c r="B7" t="s" s="6">
-        <v>114</v>
-      </c>
-      <c r="C7" t="s" s="14">
-        <v>125</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
@@ -3800,7 +3779,7 @@
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
       <c r="N7" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="O7" s="3"/>
       <c r="P7" s="3"/>
@@ -3816,14 +3795,14 @@
       <c r="Z7" s="3"/>
     </row>
     <row r="8" ht="13.55" customHeight="1">
-      <c r="A8" t="s" s="13">
-        <v>69</v>
-      </c>
-      <c r="B8" t="s" s="6">
-        <v>114</v>
-      </c>
-      <c r="C8" t="s" s="14">
-        <v>126</v>
+      <c r="A8" t="s" s="2">
+        <v>68</v>
+      </c>
+      <c r="B8" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="C8" t="s" s="2">
+        <v>125</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
@@ -3836,7 +3815,7 @@
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
       <c r="N8" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="O8" s="3"/>
       <c r="P8" s="3"/>
@@ -3852,14 +3831,14 @@
       <c r="Z8" s="3"/>
     </row>
     <row r="9" ht="13.55" customHeight="1">
-      <c r="A9" t="s" s="13">
-        <v>82</v>
-      </c>
-      <c r="B9" t="s" s="6">
-        <v>114</v>
-      </c>
-      <c r="C9" t="s" s="14">
-        <v>127</v>
+      <c r="A9" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="B9" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="C9" t="s" s="2">
+        <v>126</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -3872,7 +3851,7 @@
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
       <c r="N9" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="O9" s="3"/>
       <c r="P9" s="3"/>
@@ -3888,14 +3867,14 @@
       <c r="Z9" s="3"/>
     </row>
     <row r="10" ht="13.55" customHeight="1">
-      <c r="A10" t="s" s="13">
-        <v>62</v>
-      </c>
-      <c r="B10" t="s" s="6">
-        <v>114</v>
-      </c>
-      <c r="C10" t="s" s="14">
-        <v>128</v>
+      <c r="A10" t="s" s="2">
+        <v>61</v>
+      </c>
+      <c r="B10" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="C10" t="s" s="2">
+        <v>127</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
@@ -3908,7 +3887,7 @@
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
       <c r="N10" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
@@ -3924,14 +3903,14 @@
       <c r="Z10" s="3"/>
     </row>
     <row r="11" ht="13.55" customHeight="1">
-      <c r="A11" t="s" s="13">
-        <v>94</v>
-      </c>
-      <c r="B11" t="s" s="6">
-        <v>114</v>
-      </c>
-      <c r="C11" t="s" s="14">
-        <v>129</v>
+      <c r="A11" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="B11" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="C11" t="s" s="2">
+        <v>128</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
@@ -3944,7 +3923,7 @@
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
       <c r="N11" t="s" s="2">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
@@ -3973,15 +3952,15 @@
   <dimension ref="A1:Z19"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="25.25" style="15" customWidth="1"/>
-    <col min="2" max="2" width="24.5" style="15" customWidth="1"/>
-    <col min="3" max="3" width="51.7891" style="15" customWidth="1"/>
-    <col min="4" max="4" width="22.3516" style="15" customWidth="1"/>
-    <col min="5" max="5" width="54.3516" style="15" customWidth="1"/>
-    <col min="6" max="6" width="25" style="15" customWidth="1"/>
-    <col min="7" max="7" width="28.6719" style="15" customWidth="1"/>
-    <col min="8" max="26" width="8.85156" style="15" customWidth="1"/>
-    <col min="27" max="16384" width="8.85156" style="15" customWidth="1"/>
+    <col min="1" max="1" width="20.8516" style="12" customWidth="1"/>
+    <col min="2" max="2" width="24.5" style="12" customWidth="1"/>
+    <col min="3" max="3" width="27.8516" style="12" customWidth="1"/>
+    <col min="4" max="4" width="22.3516" style="12" customWidth="1"/>
+    <col min="5" max="5" width="54.3516" style="12" customWidth="1"/>
+    <col min="6" max="6" width="25" style="12" customWidth="1"/>
+    <col min="7" max="7" width="28.6719" style="12" customWidth="1"/>
+    <col min="8" max="26" width="8.85156" style="12" customWidth="1"/>
+    <col min="27" max="16384" width="8.85156" style="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.55" customHeight="1">
@@ -3995,16 +3974,16 @@
         <v>29</v>
       </c>
       <c r="D1" t="s" s="2">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E1" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="F1" t="s" s="2">
         <v>131</v>
       </c>
-      <c r="F1" t="s" s="2">
+      <c r="G1" t="s" s="2">
         <v>132</v>
-      </c>
-      <c r="G1" t="s" s="2">
-        <v>133</v>
       </c>
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
@@ -4031,18 +4010,22 @@
         <v>40</v>
       </c>
       <c r="B2" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="C2" t="s" s="2">
         <v>134</v>
       </c>
-      <c r="C2" t="s" s="2">
+      <c r="D2" t="s" s="2">
         <v>135</v>
       </c>
-      <c r="D2" t="s" s="2">
+      <c r="E2" t="s" s="2">
         <v>136</v>
       </c>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="F2" t="s" s="2">
+        <v>137</v>
+      </c>
       <c r="G2" t="s" s="2">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
@@ -4066,21 +4049,25 @@
     </row>
     <row r="3" ht="13.55" customHeight="1">
       <c r="A3" t="s" s="2">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C3" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="D3" t="s" s="2">
+        <v>139</v>
+      </c>
+      <c r="E3" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="F3" t="s" s="2">
         <v>137</v>
       </c>
-      <c r="D3" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
       <c r="G3" t="s" s="2">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
@@ -4104,21 +4091,25 @@
     </row>
     <row r="4" ht="13.55" customHeight="1">
       <c r="A4" t="s" s="2">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>140</v>
-      </c>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
+        <v>141</v>
+      </c>
+      <c r="E4" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="F4" t="s" s="2">
+        <v>137</v>
+      </c>
       <c r="G4" t="s" s="2">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
@@ -4142,21 +4133,25 @@
     </row>
     <row r="5" ht="13.55" customHeight="1">
       <c r="A5" t="s" s="2">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>142</v>
-      </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
+        <v>143</v>
+      </c>
+      <c r="E5" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="F5" t="s" s="2">
+        <v>137</v>
+      </c>
       <c r="G5" t="s" s="2">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
@@ -4180,21 +4175,25 @@
     </row>
     <row r="6" ht="13.55" customHeight="1">
       <c r="A6" t="s" s="2">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>145</v>
-      </c>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+        <v>146</v>
+      </c>
+      <c r="E6" t="s" s="2">
+        <v>147</v>
+      </c>
+      <c r="F6" t="s" s="2">
+        <v>148</v>
+      </c>
       <c r="G6" t="s" s="2">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
@@ -4218,21 +4217,25 @@
     </row>
     <row r="7" ht="13.55" customHeight="1">
       <c r="A7" t="s" s="2">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>148</v>
-      </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
+        <v>151</v>
+      </c>
+      <c r="E7" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="F7" t="s" s="2">
+        <v>153</v>
+      </c>
       <c r="G7" t="s" s="2">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
@@ -4256,21 +4259,25 @@
     </row>
     <row r="8" ht="13.55" customHeight="1">
       <c r="A8" t="s" s="2">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C8" t="s" s="2">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>150</v>
-      </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
+        <v>155</v>
+      </c>
+      <c r="E8" t="s" s="2">
+        <v>156</v>
+      </c>
+      <c r="F8" t="s" s="2">
+        <v>157</v>
+      </c>
       <c r="G8" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
@@ -4294,21 +4301,25 @@
     </row>
     <row r="9" ht="13.55" customHeight="1">
       <c r="A9" t="s" s="2">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C9" t="s" s="2">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>152</v>
-      </c>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
+        <v>159</v>
+      </c>
+      <c r="E9" t="s" s="2">
+        <v>156</v>
+      </c>
+      <c r="F9" t="s" s="2">
+        <v>160</v>
+      </c>
       <c r="G9" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
@@ -4332,21 +4343,25 @@
     </row>
     <row r="10" ht="13.55" customHeight="1">
       <c r="A10" t="s" s="2">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>154</v>
-      </c>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
+        <v>162</v>
+      </c>
+      <c r="E10" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="F10" t="s" s="2">
+        <v>164</v>
+      </c>
       <c r="G10" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
@@ -4370,21 +4385,25 @@
     </row>
     <row r="11" ht="13.55" customHeight="1">
       <c r="A11" t="s" s="2">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C11" t="s" s="2">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>156</v>
-      </c>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
+        <v>166</v>
+      </c>
+      <c r="E11" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="F11" t="s" s="2">
+        <v>164</v>
+      </c>
       <c r="G11" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
@@ -4408,21 +4427,25 @@
     </row>
     <row r="12" ht="13.55" customHeight="1">
       <c r="A12" t="s" s="2">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C12" t="s" s="2">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="D12" t="s" s="2">
-        <v>158</v>
-      </c>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
+        <v>168</v>
+      </c>
+      <c r="E12" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="F12" t="s" s="2">
+        <v>164</v>
+      </c>
       <c r="G12" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
@@ -4446,21 +4469,25 @@
     </row>
     <row r="13" ht="13.55" customHeight="1">
       <c r="A13" t="s" s="2">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C13" t="s" s="2">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="D13" t="s" s="2">
-        <v>160</v>
-      </c>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
+        <v>170</v>
+      </c>
+      <c r="E13" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="F13" t="s" s="2">
+        <v>164</v>
+      </c>
       <c r="G13" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
@@ -4484,21 +4511,25 @@
     </row>
     <row r="14" ht="13.55" customHeight="1">
       <c r="A14" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C14" t="s" s="2">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="D14" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
+        <v>172</v>
+      </c>
+      <c r="E14" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="F14" t="s" s="2">
+        <v>164</v>
+      </c>
       <c r="G14" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
@@ -4522,21 +4553,25 @@
     </row>
     <row r="15" ht="13.55" customHeight="1">
       <c r="A15" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="D15" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="E15" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="F15" t="s" s="2">
         <v>164</v>
       </c>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
       <c r="G15" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
@@ -4560,21 +4595,25 @@
     </row>
     <row r="16" ht="13.55" customHeight="1">
       <c r="A16" t="s" s="2">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C16" t="s" s="2">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="D16" t="s" s="2">
-        <v>166</v>
-      </c>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
+        <v>177</v>
+      </c>
+      <c r="E16" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="F16" t="s" s="2">
+        <v>164</v>
+      </c>
       <c r="G16" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
@@ -4598,21 +4637,25 @@
     </row>
     <row r="17" ht="13.55" customHeight="1">
       <c r="A17" t="s" s="2">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C17" t="s" s="2">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="D17" t="s" s="2">
-        <v>168</v>
-      </c>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
+        <v>179</v>
+      </c>
+      <c r="E17" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="F17" t="s" s="2">
+        <v>164</v>
+      </c>
       <c r="G17" t="s" s="2">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
@@ -4636,21 +4679,25 @@
     </row>
     <row r="18" ht="13.55" customHeight="1">
       <c r="A18" t="s" s="2">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C18" t="s" s="2">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="D18" t="s" s="2">
-        <v>170</v>
-      </c>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
+        <v>181</v>
+      </c>
+      <c r="E18" t="s" s="2">
+        <v>182</v>
+      </c>
+      <c r="F18" t="s" s="2">
+        <v>148</v>
+      </c>
       <c r="G18" t="s" s="2">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
@@ -4674,21 +4721,25 @@
     </row>
     <row r="19" ht="13.55" customHeight="1">
       <c r="A19" t="s" s="2">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C19" t="s" s="2">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="D19" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
+        <v>184</v>
+      </c>
+      <c r="E19" t="s" s="2">
+        <v>185</v>
+      </c>
+      <c r="F19" t="s" s="2">
+        <v>153</v>
+      </c>
       <c r="G19" t="s" s="2">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
@@ -4724,8 +4775,8 @@
   <dimension ref="A1:Z10"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="26" width="8.85156" style="16" customWidth="1"/>
-    <col min="27" max="16384" width="8.85156" style="16" customWidth="1"/>
+    <col min="1" max="26" width="8.85156" style="13" customWidth="1"/>
+    <col min="27" max="16384" width="8.85156" style="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.55" customHeight="1">
@@ -4739,10 +4790,10 @@
         <v>29</v>
       </c>
       <c r="D1" t="s" s="2">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E1" t="s" s="2">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
@@ -5032,8 +5083,8 @@
   <dimension ref="A1:Z10"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="26" width="8.85156" style="17" customWidth="1"/>
-    <col min="27" max="16384" width="8.85156" style="17" customWidth="1"/>
+    <col min="1" max="26" width="8.85156" style="14" customWidth="1"/>
+    <col min="27" max="16384" width="8.85156" style="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.55" customHeight="1">
@@ -5044,40 +5095,40 @@
         <v>28</v>
       </c>
       <c r="C1" t="s" s="2">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="D1" t="s" s="2">
         <v>29</v>
       </c>
       <c r="E1" t="s" s="2">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="F1" t="s" s="2">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="G1" t="s" s="2">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="H1" t="s" s="2">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="I1" t="s" s="2">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="J1" t="s" s="2">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="K1" t="s" s="2">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="L1" t="s" s="2">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="M1" t="s" s="2">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="N1" t="s" s="2">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="O1" s="3"/>
       <c r="P1" s="3"/>
@@ -5358,8 +5409,8 @@
   <dimension ref="A1:Z10"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="26" width="8.85156" style="18" customWidth="1"/>
-    <col min="27" max="16384" width="8.85156" style="18" customWidth="1"/>
+    <col min="1" max="26" width="8.85156" style="15" customWidth="1"/>
+    <col min="27" max="16384" width="8.85156" style="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.55" customHeight="1">
@@ -5370,34 +5421,34 @@
         <v>28</v>
       </c>
       <c r="C1" t="s" s="2">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="D1" t="s" s="2">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="E1" t="s" s="2">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="F1" t="s" s="2">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="G1" t="s" s="2">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="H1" t="s" s="2">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="I1" t="s" s="2">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="J1" t="s" s="2">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="K1" t="s" s="2">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="L1" t="s" s="2">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="M1" s="3"/>
       <c r="N1" s="3"/>

</xml_diff>